<commit_message>
bug in storing win probs
</commit_message>
<xml_diff>
--- a/04_tournaments/2025_ncaa_tournament_seeds.xlsx
+++ b/04_tournaments/2025_ncaa_tournament_seeds.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zhostetl\Documents\11_CBB\99_git\NC2A-CBB\04_tournaments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94EC116-4F98-4275-BAEF-5E5938E014A3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{40FD0C11-57AE-4CFB-B9A3-205D1751674A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{B2332335-16DB-4434-86FE-47B54B5B1C81}"/>
   </bookViews>
@@ -182,9 +182,6 @@
     <t>Liberty Flames</t>
   </si>
   <si>
-    <t>Seatle, WA</t>
-  </si>
-  <si>
     <t>VCU Rams</t>
   </si>
   <si>
@@ -266,9 +263,6 @@
     <t>Denver, CO</t>
   </si>
   <si>
-    <t>Clevand, OH</t>
-  </si>
-  <si>
     <t>Wichita, KS</t>
   </si>
   <si>
@@ -279,6 +273,12 @@
   </si>
   <si>
     <t>Milwaukee, WI</t>
+  </si>
+  <si>
+    <t>Seattle, WA</t>
+  </si>
+  <si>
+    <t>Cleveland, OH</t>
   </si>
 </sst>
 </file>
@@ -756,7 +756,7 @@
         <v>3</v>
       </c>
       <c r="E6" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -773,7 +773,7 @@
         <v>3</v>
       </c>
       <c r="E7" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
@@ -790,7 +790,7 @@
         <v>4</v>
       </c>
       <c r="E8" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -807,7 +807,7 @@
         <v>4</v>
       </c>
       <c r="E9" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
@@ -824,12 +824,12 @@
         <v>5</v>
       </c>
       <c r="E10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B11">
         <v>11</v>
@@ -841,7 +841,7 @@
         <v>5</v>
       </c>
       <c r="E11" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
@@ -858,12 +858,12 @@
         <v>6</v>
       </c>
       <c r="E12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B13">
         <v>14</v>
@@ -875,7 +875,7 @@
         <v>6</v>
       </c>
       <c r="E13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -892,12 +892,12 @@
         <v>7</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B15">
         <v>10</v>
@@ -909,7 +909,7 @@
         <v>7</v>
       </c>
       <c r="E15" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -926,12 +926,12 @@
         <v>8</v>
       </c>
       <c r="E16" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B17">
         <v>15</v>
@@ -943,7 +943,7 @@
         <v>8</v>
       </c>
       <c r="E17" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
@@ -965,7 +965,7 @@
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B19">
         <v>16</v>
@@ -999,7 +999,7 @@
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B21">
         <v>9</v>
@@ -1016,7 +1016,7 @@
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B22">
         <v>5</v>
@@ -1028,7 +1028,7 @@
         <v>3</v>
       </c>
       <c r="E22" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
@@ -1045,12 +1045,12 @@
         <v>3</v>
       </c>
       <c r="E23" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24">
         <v>4</v>
@@ -1062,7 +1062,7 @@
         <v>4</v>
       </c>
       <c r="E24" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
@@ -1079,12 +1079,12 @@
         <v>4</v>
       </c>
       <c r="E25" t="s">
-        <v>48</v>
+        <v>79</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B26">
         <v>6</v>
@@ -1096,7 +1096,7 @@
         <v>5</v>
       </c>
       <c r="E26" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -1113,7 +1113,7 @@
         <v>5</v>
       </c>
       <c r="E27" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
@@ -1130,12 +1130,12 @@
         <v>6</v>
       </c>
       <c r="E28" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B29">
         <v>14</v>
@@ -1147,7 +1147,7 @@
         <v>6</v>
       </c>
       <c r="E29" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1164,12 +1164,12 @@
         <v>7</v>
       </c>
       <c r="E30" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B31">
         <v>10</v>
@@ -1181,12 +1181,12 @@
         <v>7</v>
       </c>
       <c r="E31" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="B32">
         <v>2</v>
@@ -1198,12 +1198,12 @@
         <v>8</v>
       </c>
       <c r="E32" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="B33">
         <v>15</v>
@@ -1215,7 +1215,7 @@
         <v>8</v>
       </c>
       <c r="E33" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
@@ -1232,12 +1232,12 @@
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="B35">
         <v>16</v>
@@ -1249,12 +1249,12 @@
         <v>1</v>
       </c>
       <c r="E35" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="B36">
         <v>8</v>
@@ -1266,7 +1266,7 @@
         <v>2</v>
       </c>
       <c r="E36" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -1283,12 +1283,12 @@
         <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B38">
         <v>5</v>
@@ -1300,12 +1300,12 @@
         <v>3</v>
       </c>
       <c r="E38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B39">
         <v>12</v>
@@ -1317,7 +1317,7 @@
         <v>3</v>
       </c>
       <c r="E39" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
@@ -1334,7 +1334,7 @@
         <v>4</v>
       </c>
       <c r="E40" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -1351,12 +1351,12 @@
         <v>4</v>
       </c>
       <c r="E41" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B42">
         <v>6</v>
@@ -1368,7 +1368,7 @@
         <v>5</v>
       </c>
       <c r="E42" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -1385,7 +1385,7 @@
         <v>5</v>
       </c>
       <c r="E43" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
@@ -1402,12 +1402,12 @@
         <v>6</v>
       </c>
       <c r="E44" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B45">
         <v>14</v>
@@ -1419,7 +1419,7 @@
         <v>6</v>
       </c>
       <c r="E45" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
@@ -1436,7 +1436,7 @@
         <v>7</v>
       </c>
       <c r="E46" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
@@ -1453,7 +1453,7 @@
         <v>7</v>
       </c>
       <c r="E47" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
@@ -1470,12 +1470,12 @@
         <v>8</v>
       </c>
       <c r="E48" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B49">
         <v>15</v>
@@ -1487,7 +1487,7 @@
         <v>8</v>
       </c>
       <c r="E49" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
@@ -1504,12 +1504,12 @@
         <v>1</v>
       </c>
       <c r="E50" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B51">
         <v>16</v>
@@ -1521,7 +1521,7 @@
         <v>1</v>
       </c>
       <c r="E51" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -1538,12 +1538,12 @@
         <v>2</v>
       </c>
       <c r="E52" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B53">
         <v>9</v>
@@ -1555,7 +1555,7 @@
         <v>2</v>
       </c>
       <c r="E53" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -1572,7 +1572,7 @@
         <v>3</v>
       </c>
       <c r="E54" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
@@ -1589,7 +1589,7 @@
         <v>3</v>
       </c>
       <c r="E55" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
@@ -1606,12 +1606,12 @@
         <v>4</v>
       </c>
       <c r="E56" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B57">
         <v>13</v>
@@ -1623,7 +1623,7 @@
         <v>4</v>
       </c>
       <c r="E57" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
@@ -1640,7 +1640,7 @@
         <v>5</v>
       </c>
       <c r="E58" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
@@ -1657,7 +1657,7 @@
         <v>5</v>
       </c>
       <c r="E59" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
@@ -1674,12 +1674,12 @@
         <v>6</v>
       </c>
       <c r="E60" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B61">
         <v>14</v>
@@ -1691,12 +1691,12 @@
         <v>6</v>
       </c>
       <c r="E61" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B62">
         <v>7</v>
@@ -1708,7 +1708,7 @@
         <v>7</v>
       </c>
       <c r="E62" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
@@ -1725,7 +1725,7 @@
         <v>7</v>
       </c>
       <c r="E63" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
@@ -1742,12 +1742,12 @@
         <v>8</v>
       </c>
       <c r="E64" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B65">
         <v>15</v>
@@ -1759,7 +1759,7 @@
         <v>8</v>
       </c>
       <c r="E65" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
   </sheetData>

</xml_diff>